<commit_message>
chore: log versioni e report giornaliero fase 2
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +38,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F6FC"/>
         <bgColor rgb="00F2F6FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,12 +104,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -471,8 +480,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -575,8 +584,51 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>v0.3.0</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>16:13:40</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Aggiunto: OpenRouterEngine (convert, suggest_topic) | Aggiunto: split_pdf/needs_split, derive_topic/slugify_topic/unique_path, classify_page/classify_pdf | Aggiunto: run_batch+BatchConfig con auto-split e progressi | Modificato: pipeline.convert — routing native/hybrid/llm, PageResult.engine | Ristrutturato: cli.main a sottocomandi convert/batch/split/gui | Aggiunto: gui/server.py + static index/style/app (GUI locale)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Fase 2: engine LLM OpenRouter, batch con rinomina argomento max 10 char, partizionatore PDF per limiti pagine/MB, GUI HTML/JS/CSS con banner avanzamento</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/engines/openrouter.py; src/pdf2md_pro/engines/base.py; src/pdf2md_pro/core/splitter.py; src/pdf2md_pro/core/naming.py; src/pdf2md_pro/core/classifier.py; src/pdf2md_pro/core/batch.py; src/pdf2md_pro/core/pipeline.py; src/pdf2md_pro/cli.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/style.css; src/pdf2md_pro/gui/static/app.js</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni aggiornato
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -627,8 +627,51 @@
       </c>
       <c r="I3" s="3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>v0.4.0</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>16:21:31</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Claude Fable 5</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto: make_llm_engine/ensure_ollama — provider glmocr (Ollama locale, default) e openrouter | Modificato: OpenRouterEngine — api_url/provider parametrici, chiave opzionale | Modificato: BatchConfig — provider/ollama_url | Modificato: GUI — selettore provider, campi Ollama, datalist nemotron</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>GLM-OCR locale via Ollama come modello LLM predefinito, OpenRouter configurabile con modelli tipo nemotron free</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/engines/openrouter.py; src/pdf2md_pro/core/batch.py; src/pdf2md_pro/cli.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/app.js; tests/test_openrouter.py</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
+  <autoFilter ref="A1:I4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni fix GUI
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -756,8 +756,51 @@
       </c>
       <c r="I6" s="2" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>v0.6.1</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>20:54:49</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Corretto</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Corretto: GUI aperta come file:// — guardia OFFLINE + fetchErrorText sostituiscono 'Failed to fetch' con istruzione 'pdf2md gui' | Aggiunto: _clean_path (server) — de-escape backslash e apici nei percorsi incollati con spazi | Corretto: messaggi errore analyze/split/convert/pick</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>errore nel partizionare i file: Failed to fetch aprendo GUI come file locale e percorsi con spazi escaped</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/gui/static/app.js; src/pdf2md_pro/gui/server.py; tests/test_gui_server.py</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni launcher GUI
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -799,8 +799,51 @@
       </c>
       <c r="I7" s="3" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>v0.7.0</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>21:22:40</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto: avvia-gui.command — launcher doppio-click (Terminale + server + browser) | Modificato: serve() — gestione OSError porta occupata con messaggio chiaro, print flush, messaggio stop | Modificato: README sezione GUI e nota ERR_CONNECTION_REFUSED</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>ERR_CONNECTION_REFUSED su localhost: server GUI non avviato; serve modo semplice per lanciarlo</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>avvia-gui.command; src/pdf2md_pro/gui/server.py; README.md</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
+  <autoFilter ref="A1:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni persistenza GUI
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -842,8 +842,51 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>v0.8.0</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>21:26:51</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Aggiunto: persistenza impostazioni GUI in localStorage (saveConfig/restoreConfig) — cartelle, motore, provider, limiti salvati e ricaricati a ogni avvio | Aggiunto: checkbox 'Ricorda la chiave' — chiave API salvata solo con opt-in esplicito | Modificato: syncConditionalFields riusato al restore</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>impostate le configurazioni devono essere salvate automaticamente in tutti gli accessi successivi</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/gui/static/app.js; src/pdf2md_pro/gui/static/index.html</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni servizio always-on
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -885,8 +885,51 @@
       </c>
       <c r="I9" s="3" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>v0.9.0</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>21:33:01</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto: installa-servizio.command / ferma-servizio.command — LaunchAgent macOS, GUI sempre attiva su 8347, avvio al login, riavvio automatico | Aggiunto: flag 'pdf2md gui --no-open' e serve(open_browser) — il servizio non apre il browser a ogni login</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>ERR_CONNECTION_REFUSED ricorrente: il server GUI non resta attivo; serve modo per averlo sempre disponibile</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>installa-servizio.command; ferma-servizio.command; src/pdf2md_pro/cli.py; src/pdf2md_pro/gui/server.py; README.md</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:I10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni filtro AppleDouble
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -928,8 +928,51 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>v0.9.1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>21:35:31</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Corretto</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Aggiunto: list_pdfs — helper condiviso che esclude file nascosti e AppleDouble macOS (._nome.pdf) | Corretto: analyze_folder/split_folder/run_batch usano list_pdfs, niente più errori 'Failed to open ._*.pdf' su drive esterni exFAT</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>errori 'Failed to open ._*.pdf': file AppleDouble di macOS su drive esterno vengono presi come PDF</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/core/splitter.py; src/pdf2md_pro/core/batch.py; tests/test_splitter.py</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni pausa/stop
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -971,8 +971,51 @@
       </c>
       <c r="I11" s="3" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>v0.10.0</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>05:51:08</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto: JobControl (pausa/riprendi/stop) e run_batch(control=...) — pausa tra file, stop dopo file corrente | Aggiunto: endpoint /api/pause /api/resume /api/stop e pulsanti banner GUI | Modificato: etichette motore Nativo/Ibrido/LLM chiariscono che GLM-OCR si usa in Ibrido e LLM totale</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>aggiungere pausa/sospensione conversione PDF-&gt;MD; chiarire in quale modalità si usa GLM-OCR</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/core/batch.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/app.js; src/pdf2md_pro/gui/static/style.css; tests/test_batch.py</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
+  <autoFilter ref="A1:I12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni nome originale
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1014,8 +1014,51 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>v0.10.1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>05:55:03</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Modificato</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Modificato: _deliver/BatchConfig — il md conserva il nome del PDF originale di default (rename_by_topic=False) | Aggiunto: opzione GUI 'Rinomina per argomento' (default off) e persistenza checkbox rename-topic</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>il file md deve mantenere lo stesso titolo del file pdf originale</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/core/batch.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/app.js; tests/test_batch.py</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
+  <autoFilter ref="A1:I13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni selezione file + badge versione
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1057,8 +1057,51 @@
       </c>
       <c r="I13" s="3" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>v0.11.0</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>06:15:16</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto: BatchConfig.only_files + filtro run_batch — convertire solo file selezionati | Aggiunto: endpoint /api/list-pdfs e /api/version | Aggiunto: GUI selezione file (checklist tutti/nessuno) e badge versione log accanto al titolo | Aggiunto: __version__ pacchetto</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>prevedere selezione dei soli file da convertire in md; aggiungere versione log accanto al titolo</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/__init__.py; src/pdf2md_pro/core/batch.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/app.js; src/pdf2md_pro/gui/static/style.css; tests/test_batch.py</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:I14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni partizione in loco
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1100,8 +1100,51 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>v0.11.1</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>06:31:20</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Modificato</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Modificato: split_folder ora lavora in loco (niente out_dir) — parti restano nella cartella elaborata | Aggiunto: partition_in_place + costante INTERI_DIR — originali spezzati spostati in interi/ | Modificato: server _run_split, CLI split (rimosso -o), GUI (rimosso campo cartella uscita, passo 3 converte la cartella, interi/ ignorata)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>la partizione deve lasciare le parti nella cartella elaborata e spostare gli originali partizionati in una cartella chiamata interi</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/core/splitter.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/cli.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/app.js; src/pdf2md_pro/__init__.py; tests/test_splitter.py</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I14"/>
+  <autoFilter ref="A1:I15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: log versioni interi-dir
</commit_message>
<xml_diff>
--- a/archivio_versioni.xlsx
+++ b/archivio_versioni.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog SemVer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changelog SemVer'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1143,8 +1143,51 @@
       </c>
       <c r="I15" s="3" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>v0.12.0</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>06:50:01</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Claude Opus 4.8</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Aggiunto: parametro interi_dir in partition_in_place/split_folder — cartella archivio originali configurabile (default interi/) | Aggiunto: --interi-dir CLI, payload interi_dir server, campo GUI 'Cartella archivio degli originali' con Sfoglia e persistenza</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>nella partizione poter scegliere la cartella dove archiviare i file interi dopo averli partizionati</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>src/pdf2md_pro/core/splitter.py; src/pdf2md_pro/gui/server.py; src/pdf2md_pro/cli.py; src/pdf2md_pro/gui/static/index.html; src/pdf2md_pro/gui/static/app.js; src/pdf2md_pro/__init__.py; tests/test_splitter.py</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I15"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>